<commit_message>
new recommendation ws notification
</commit_message>
<xml_diff>
--- a/backend/Basic data.xlsx
+++ b/backend/Basic data.xlsx
@@ -23,8 +23,8 @@
     <t>ru</t>
   </si>
   <si>
-    <t>The Likes app allows you to find new connections based on your personal values.
-I'm working from the following assumption.
+    <t>The Likes is an application for finding people with same values.
+I proceed from the following assumption.
 1. Friendship begins and is maintained not by logic, but by emotion. We can be friends with someone who doesn't share our values — and not notice it amidst the positive emotions.
 2. Over time (due to technological development, the spread of education, or some other reasons), people become more rational — relying less on emotions and more on logic, analysis, strategy, etc. This makes it more difficult for them to make new friends.
 3. I don't think the process of rationalization can be stopped. If we want to preserve friendship, we must learn to begin new relationships not with emotion, but on rational grounds — personal values.
@@ -52,7 +52,7 @@
 Therefore, despite the obstacles, I propose this approach.</t>
   </si>
   <si>
-    <t>The Likes позволяет найти новых знакомых на основе персональных ценностей.
+    <t>The Likes — это приложение для поиска людей со схожими ценностями.
 Я исхожу из следующего предположения.
 1. Дружба начинается и поддерживается не логикой, а эмоциями. Мы можем дружить с человеком, который не разделяет наших ценностей — и не замечать этого на фоне положительных эмоций.
 2. С течением времени (из-за технического развития, распространения образования, или ещё каких—то причин) люди становятся более рациональными — меньше полагаются на эмоции, и больше — на логику, анализ, статегию и т.п. Поэтому им становится труднее заводить новых друзей.
@@ -69,7 +69,7 @@
 5. Далее я буду употреблять термин "ценности" в следующем значении. Ценности — это термины, которые:
 • высоко-абстрактны;
 • работают как моральные ориентиры (действия, слова, мысли, решения, поведение любого человека — всегда в какой—то степени будут направлены к/от "любви", "красоты" и т.п.);
-• финально не достижимы, но их можно бесконечно эффективно преследовать (невозможно обрести всю возможную любовь во вселенной, но но всегда можно найти больше любви);
+• финально не достижимы, но их можно бесконечно эффективно преследовать (невозможно обрести всю возможную любовь во вселенной, но всегда можно найти больше любви);
 • нейтральны сами по себе, пока не организованы в иерархию (любовь сама по себе — ни хорошая, ни плохая — мы сами выбираем, в какой степени стремиться к ней / от неё — и только этот выбор создаёт иерархию — помещает любовь выше/ниже других моральных ценностей).
 6. 
 6.1. У каждого человека есть внутренняя иерархия ценностей, которая оказывает влияние на его эмоции, мысли, язык, решения и поведение и т.д. И / или:
@@ -83,21 +83,19 @@
   <si>
     <t>I offer you a set of terms denoting possible abstract values: Pleasure, Comfort, Happiness, Love, Beauty, Wealth, Status, Power, Violence, Truth, Freedom.
 In the first step, you must select components — Aspects — for each value. If you agree that a statement should be included in the value definition, check the box next to it. For example, if you agree that Beauty is (partially or completely) an objective quality, include this aspect in the definition of beauty.
-Choose your Aspects carefully. Each combination of Aspects is considered by the algorithm as an independent Value. That is, if you included the Aspect "objective quality" in Beauty, and someone else included all the same Aspects as you, but did not include "objective quality," we do not know how close or distant these two concepts are. Therefore, your Beauty and the Beauty of that other person are considered by the algorithm as Two completely different values ​​(despite the same name – Beauty).
-In the second step, distribute the Values ​​among three groups: positive, negative, and neutral. Initially, all Values ​​are in the neutral group. If, for example, you want more Beauty in reality, move it to the positive group. If, conversely, you believe there should be less Beauty, move it to the negative group. If you want neither more nor less Beauty, leave it in the neutral group. Distribute all Values ​​according to this principle.
-Positive and negative Values ​​should be arranged hierarchically, according to how you feel about them: in first place among the positive — the Value most dear to you, in second place is the next most dear, and so on. Negative Values: in last place is the most unpleasant and undesirable, in second to last is the almost most unpleasant/undesirable, and so on. Neutral values ​​do not need to be sorted — their order doesn't matter.
-This task may require considerable deliberation. It's best to make a decision when you can identify the two most desired and two least desired values. Though the values ​​can be ordered any way you like — all decisions will be taken into account — preference will be given to the first two positive and last two negative values. (Here, I'm assuming that in most cases a person have at least 2 positive and two negative values, and those values are most decisive.)
-You can change your value profile later, but frequent changes will reduce your chances of making friends.
+Important: each combination of Aspects is considered as an independent Value. That is, if you included the Aspect "objective quality" in Beauty, and someone else — not — we do not know how close or distant is your view on Beauty from the view of that other person.
+In the second step, distribute your Values ​​among three groups: positive, negative, and neutral. Initially, all Values ​​are in the neutral group. If you want more Beauty in your life, move it to the positive. If less, move it to the negative. Leave the values ​​you don't care about in the neutral group.
+Positive and negative Values ​​should be arranged hierarchically according to how you feel about them: the best at the very top, the worst at the very bottom. Neutral values ​​don't need to be sorted — their order doesn't matter.
+Though the values ​​can be ordered any way you like — all decisions will be taken into account — preference will be given to the first two positive and last two negative values. You can change Aspects and Values hierarchy later, but frequent changes will reduce chances of getting a recommendation.
 In the third step, you'll choose a statement that characterizes your overall attitude toward values.</t>
   </si>
   <si>
     <t>Предлагаю вам набор терминов, означающих возможные абстрактные ценности: Удовольствие, Комфорт, Счастье, Любовь, Красота, Богатство, Статус, Власть, Насилие, Истина, Свобода.
 На первом этапе для каждой ценности необходимо выбрать составляющие — Аспекты. Если вы согласны с тем, что утверждение должно быть включено в определение ценности, — поставьте галочку рядом с ним. Например, если вы согласны, что Красота — это (частично или полностью) объективное качество — включите этот аспект в опредение красоты.
-Внимательно выбирайте Аспекты. Каждая комбинация Аспектов рассматривается алгоритмом как самостоятельная Ценность. То есть, если вы включили Аспект "объективное качество" в Красоту, а кто—то другой включил в Красоту все те же Аспекты, что и вы, но не включил "объективное качество" — мы не знаем, насколько близки или далеки эти два понятия. Поэтому, ваша Красота, и Красота того второго человека рассматриваются алгоритмом как две совершенно разные ценнсти (несмотря на одинаковое название — Красота).
-На втором этапе распределите Цености между тремя группами: позитивные, негативные и нейтральные. Вначале все Ценности находятся в нейтральной группе. Если, например, вы хотите, чтобы в реальности было больше Красоты, — переместите её в группу позитивных. Если, наоборот, считаете, что Красоты должно быть меньше — переместите в группу негативных. Если же не хотите ни больше, ни меньше Красоты — оставьте её в нейтральной группе. По такому принципу распределите все Ценности.
-Позитивные и негативные Ценности нужно располжить иерархически, в соответствии с тем, как вы к ним относитесть: на первом месте среди позитивных — самую дорогую для вас Ценность, на втором месте — пости самую дорогую, и так далее. Негативные Ценности: на последнем месте самое неприятное и нежеланное, на предпоследнем — почти самое неприятное/нежеланное, и так далее. Нейтральные ценнсти сортировать не нужно — их порядок не имеет значения.
-Эта задача может потребовать длительных размышлений. Желательно принять решение тогда, когда сможете выбрать две самые желанные и две самые нежеланные Ценности. Хотя Ценности можно распределить как угодно — и все решения будут учтены — наибольший "вес" будут иметь две первые позитивные и две последние негативные Ценности. (Здесь я предполагаю, что в большинстве случаев у человека есть по крайней мере 2 позитивных и 2 негативных ценности, и эти ценности являются решающими.)
-Ценностный профиль можно будет изменить позже, но частые изменения понизят шансы найти друзей.
+Важно: каждая комбинация Аспектов рассматривается как самостоятельная Ценность. То есть, если вы включили Аспект "объективное качество" в Красоту, а кто-то другой — нет — то мы не знаем, насколько близко или далеко ваше понимание красоты от того, как её понимает тот другой человек.
+На втором этапе распределите Цености между тремя группами: позитивные, негативные и нейтральные. Вначале все Ценности находятся в нейтральной группе. Если вы хотите больше Красоты в своей жизни — переместите её позитивные. Если меньше — в негативные. В нейтральной группе оставьте то, что вам безразлично.
+Позитивные и негативные Ценности нужно располжить иерархически, в соответствии с тем, как вы к ним относитесть: самое хорошее - на самом верху, самое плохое - в самом низу. Нейтральные ценнсти сортировать не нужно — их порядок не имеет значения.
+Хотя Ценности можно распределить как угодно — и все решения будут учтены — наибольший "вес" будут иметь две первые позитивные и две последние негативные Ценности. Аспекты и иерархию Ценностей можно будет изменить позже, но частые изменения понизят шансы получить рекоммендацию.
 На третьем этапе выберете утверждение, которое характеризует ваше отношение к ценностям в целом.</t>
   </si>
   <si>
@@ -446,10 +444,10 @@
     <t>через манипуляцию</t>
   </si>
   <si>
-    <t>I think power can operate through manipulation.</t>
+    <t>I think power can operate through manipulation/pressure.</t>
   </si>
   <si>
-    <t>Я думаю, что власть может действовать через манипуляцию.</t>
+    <t>Я думаю, что власть может действовать через манипуляцию/давление.</t>
   </si>
   <si>
     <t>may appear as physical harm</t>

</xml_diff>